<commit_message>
Update the OTH-AT status workbook with the OTH Platform AWS results
The AWS rows, summary counts, decisions and follow-ups now reflect the
2026-10-06 rebuild and board tests; the comparison workbook reads the
updated status directly (OTH 66 rows, 55 verified).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/doc/M2M_vs_OTH_Comparison.xlsx
+++ b/doc/M2M_vs_OTH_Comparison.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\SVN\01.ESP32\OTH_ESP32_C3\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crowm\AppData\Local\Temp\claude\C--Dev-PRJ-01-ESP32-ESP32-C3\a9c7ea1d-0f66-4b51-816d-e983995d9ece\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C08A438-4933-4B04-AC23-BC6F35F6423E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D74B6B-5DC7-4F6C-8BEF-0BA08230E09F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6885" yWindow="1305" windowWidth="32475" windowHeight="18885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'M2M 명령 결과'!$A$4:$G$70</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'OTH Platform 시험'!$A$4:$F$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'OTH 명령 결과'!$A$4:$F$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'OTH 명령 결과'!$A$4:$F$70</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기능 비교'!$A$4:$H$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">미검증·추후!$A$3:$D$18</definedName>
   </definedNames>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1294" uniqueCount="742">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1300" uniqueCount="744">
   <si>
     <t>M2M-AT / OTH-AT 기능 구현 비교 및 시험 결과</t>
   </si>
@@ -92,7 +92,7 @@
     <t>합계</t>
   </si>
   <si>
-    <t>※ M2M 66건(Ch.2~6 + 프로젝트 추가 명령), OTH는 명령 묶음 단위 행. OTH AWS 볼륨은 2026-10-06 재구현 결과(추가 명령 포함).</t>
+    <t>※ M2M 66건(Ch.2~6 + 프로젝트 추가 명령), OTH 66행(명령 묶음 단위, AWS 볼륨은 2026-10-06 OTH Platform 결과 포함).</t>
   </si>
   <si>
     <t>OTH Platform 시험 (2026-10-06)</t>
@@ -1379,7 +1379,7 @@
     <t>OTH-AT 명령별 구현/시험 결과</t>
   </si>
   <si>
-    <t>출처: OTH_ESP32_C3/doc/OTH-AT_Command_Status.xlsx (2026-10-05) + AWS 볼륨은 2026-10-06 OTH Platform 재구현 결과로 교체</t>
+    <t>출처: OTH_ESP32_C3/doc/OTH-AT_Command_Status.xlsx (2026-10-06, AWS 볼륨은 OTH Platform 재구현 결과)</t>
   </si>
   <si>
     <t>문서</t>
@@ -1790,424 +1790,430 @@
     <t>공용</t>
   </si>
   <si>
+    <t>AWS_GET</t>
+  </si>
+  <si>
+    <t>cmd_oth_aws.c</t>
+  </si>
+  <si>
+    <t>0 엔드포인트, 1 포트, 2 클라이언트ID(MAC, 인증 후 MAC_토큰), 3 인증서버, 4/5 RootCA URL, 6 지역, 7 토큰, 10 MCU 버전, 11 MCU 체크섬. 미설정 null</t>
+  </si>
+  <si>
+    <t>AWS_SEND</t>
+  </si>
+  <si>
+    <t>header/values 봉투, apiGroup 자동(A1x 001~A14x 004, A5xx 005). A100/A102는 Conn, 그 외 Event 토픽, QoS1. A100은 연결 절차 재시작. 미연결 SEND ERROR 2</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>AWS_IND</t>
+  </si>
+  <si>
+    <t>CONFIG~CONNECT OK 0, DISCONNECT ERROR 2, SEND OK, CERTIFICATE ERROR 112 확인. 실패 시 60초 뒤 재시도</t>
+  </si>
+  <si>
+    <t>AWS_RECV</t>
+  </si>
+  <si>
+    <t>Control 토픽 수신 -&gt; attributes(없으면 values 필드 평탄화). deviceId 불일치 폐기. 모의 클라우드(broker.emqx.io)로 확인, 실서버 미시험</t>
+  </si>
+  <si>
+    <t>AWS_SET (OTH Platform 추가)</t>
+  </si>
+  <si>
+    <t>개발용. 인덱스 0/1/3-7 기록, null=삭제. 인증서버/토큰 변경 시 저장 인증서 폐기, RootCA URL 변경 시 RootCA 폐기</t>
+  </si>
+  <si>
+    <t>MCU_READY (OTH Platform 추가)</t>
+  </si>
+  <si>
+    <t>호스트 MCU 버전 -&gt; AWS_GET 10, A100/A500 V02, 페어링 장치정보</t>
+  </si>
+  <si>
+    <t>MOTA_START / MOTA_READY / MOTA_DATA / MOTA_DATA_END (OTH Platform 추가)</t>
+  </si>
+  <si>
+    <t>MCU 이미지를 비활성 OTA 슬롯에 저장 후 256바이트 블록 중계(바이트 스터핑, 블록/전체 CRC32). 600바이트 이미지 CRC PC 계산값과 일치</t>
+  </si>
+  <si>
+    <t>클라우드 지시 A502 / A511 / A531 / A521 / A001 (모듈 처리)</t>
+  </si>
+  <si>
+    <t>A502 -&gt; A500 자동 응답. A511 암호화 FOTA: 해시 불일치 거부(A510 900), 정상 설치·재부팅·versionChangeW true. A521 MCU FOTA -&gt; MOTA_COUNT, 완료 후 versionChangeM true. A001 인증서 갱신 후 재접속</t>
+  </si>
+  <si>
+    <t>페어링 서버 TCP 47000 (모듈 처리)</t>
+  </si>
+  <si>
+    <t>oth_pairing.c</t>
+  </si>
+  <si>
+    <t>GEN2 프레임 DP0100-0400, AES-128 세션, SoftAP 경유 접속만 허용. 앱(또는 별도 Wi-Fi 단말) 없어 미시험</t>
+  </si>
+  <si>
+    <t>A101 등록 해지 (모듈 처리)</t>
+  </si>
+  <si>
+    <t>AWS_RECV 전달 + A102 발행 + 인증서·NV 전체 삭제 + 재부팅. 보드 AP 프로필까지 지워져 시험 보류</t>
+  </si>
+  <si>
     <t>COAP</t>
   </si>
   <si>
     <t>COAP_GET / COAP_SET / COAP_MSG</t>
   </si>
   <si>
-    <t>AWS_GET</t>
-  </si>
-  <si>
-    <t>cmd_oth_aws.c (OTH Platform)</t>
-  </si>
-  <si>
-    <t>0 엔드포인트, 1 포트, 2 클라이언트ID(MAC 또는 MAC_토큰), 3 인증서버, 4/5 RootCA URL, 6 지역, 7 토큰, 10 MCU 버전, 11 MCU 체크섬. 미설정 null</t>
-  </si>
-  <si>
-    <t>AWS_SET (추가)</t>
-  </si>
-  <si>
-    <t>cmd_oth_aws.c</t>
-  </si>
-  <si>
-    <t>개발용. 0/1/3-7 기록, null=삭제. 인증서버/토큰 변경 시 저장 인증서 폐기, RootCA URL 변경 시 RootCA 폐기</t>
-  </si>
-  <si>
-    <t>AWS_SEND</t>
-  </si>
-  <si>
-    <t>header/values 봉투, apiGroup 자동(A1x→001…A14x→004, A5xx→005). A100/A102→Conn, 그 외→Event. A100은 연결 절차 재시작. 미연결 SEND ERROR 2</t>
-  </si>
-  <si>
-    <t>MCU_READY (추가)</t>
-  </si>
-  <si>
-    <t>AWS_GET 10, A100/A500 V02, 페어링 장치정보에 사용</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>AWS_IND</t>
-  </si>
-  <si>
-    <t>CONFIG/AUTHENTICATE/CERTIFICATE/PRIVATE_KEY/ROOTCA/CONNECT OK 0, DISCONNECT ERROR 2, CERTIFICATE ERROR 112, SEND OK 확인. 실패 시 60초 재시도</t>
-  </si>
-  <si>
-    <t>AWS_RECV</t>
-  </si>
-  <si>
-    <t>Control 토픽 수신 → attributes(없으면 values 평탄화). deviceId 불일치 폐기. 모의 클라우드(broker.emqx.io)로 확인, 실서버 미시험</t>
-  </si>
-  <si>
-    <t>MOTA_START / READY / DATA / DATA_END (추가)</t>
-  </si>
-  <si>
-    <t>MCU 이미지를 비활성 OTA 슬롯에 저장 후 256바이트 블록 중계(바이트 스터핑, CRC32). 600바이트 이미지 CRC PC 계산값과 일치</t>
+    <t>OTH Platform 시험 기록 (2026-10-06, COM7 보드)</t>
+  </si>
+  <si>
+    <t>환경: ESP32-C3 보드(COM7), AP kangaps25, 모의 인증서버(PC 10.128.82.113:8080), MQTT broker.emqx.io(엔드포인트 대용), PC paho 클라이언트(클라우드 역할). 토픽 루트 OTHERS, MIB18=C545, MIB19=Air01</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>시험 항목</t>
+  </si>
+  <si>
+    <t>방법</t>
+  </si>
+  <si>
+    <t>기대 결과</t>
+  </si>
+  <si>
+    <t>실제 결과</t>
+  </si>
+  <si>
+    <t>P-01</t>
+  </si>
+  <si>
+    <t>인증 단계</t>
+  </si>
+  <si>
+    <t>모의 인증서버(PC LAN, http)</t>
+  </si>
+  <si>
+    <t>token 발급 → 클라이언트ID MAC_토큰, 인증서·키 발급/저장</t>
+  </si>
+  <si>
+    <t>AUTHENTICATE/CERTIFICATE/PRIVATE_KEY OK 0, AWS_GET 2 = 9CCC01C0C8E4_T0K3N7f3a</t>
+  </si>
+  <si>
+    <t>P-02</t>
+  </si>
+  <si>
+    <t>인증서 오류</t>
+  </si>
+  <si>
+    <t>공개 서비스(httpbin)로 인증서 없는 응답</t>
+  </si>
+  <si>
+    <t>CERTIFICATE ERROR 112</t>
+  </si>
+  <si>
+    <t>P-03</t>
+  </si>
+  <si>
+    <t>MQTT 접속</t>
+  </si>
+  <si>
+    <t>broker.emqx.io:8883 (TLS, 공개 CA 번들)</t>
+  </si>
+  <si>
+    <t>ROOTCA OK, CONNECT OK, Control 구독, A100 발행</t>
+  </si>
+  <si>
+    <t>A100 수신(V01=100, versionChange false)</t>
+  </si>
+  <si>
+    <t>P-04</t>
+  </si>
+  <si>
+    <t>저장 인증서 재사용</t>
+  </si>
+  <si>
+    <t>인증서버 정지 후 재부팅/재접속</t>
+  </si>
+  <si>
+    <t>서버 없이 접속</t>
+  </si>
+  <si>
+    <t>AUTHENTICATE~CONNECT OK 0</t>
+  </si>
+  <si>
+    <t>P-05</t>
+  </si>
+  <si>
+    <t>송신 봉투 / apiGroup</t>
+  </si>
+  <si>
+    <t>AWS_SEND=A110, A130</t>
+  </si>
+  <si>
+    <t>Event 토픽, apiGroup 001/003</t>
+  </si>
+  <si>
+    <t>일치, AWS_IND:SEND OK</t>
+  </si>
+  <si>
+    <t>P-06</t>
+  </si>
+  <si>
+    <t>수신 attributes</t>
+  </si>
+  <si>
+    <t>클라우드 A111 {attributes}</t>
+  </si>
+  <si>
+    <t>AWS_RECV:A111 23 {...}</t>
+  </si>
+  <si>
+    <t>AWS_RECV:A111 23 {"A03":"02","A04":"03"}</t>
+  </si>
+  <si>
+    <t>P-07</t>
+  </si>
+  <si>
+    <t>수신 평탄화</t>
+  </si>
+  <si>
+    <t>클라우드 A112 (attributes 없음)</t>
+  </si>
+  <si>
+    <t>values 필드를 JSON으로</t>
+  </si>
+  <si>
+    <t>AWS_RECV:A112 17 {"reqType":"all"}</t>
+  </si>
+  <si>
+    <t>P-08</t>
+  </si>
+  <si>
+    <t>타 장치 메시지</t>
+  </si>
+  <si>
+    <t>deviceId 다른 A111</t>
+  </si>
+  <si>
+    <t>폐기</t>
+  </si>
+  <si>
+    <t>호스트 출력 없음</t>
+  </si>
+  <si>
+    <t>P-09</t>
+  </si>
+  <si>
+    <t>버전 요청</t>
+  </si>
+  <si>
+    <t>클라우드 A502</t>
+  </si>
+  <si>
+    <t>모듈이 A500 자동 응답, 호스트 미전달</t>
+  </si>
+  <si>
+    <t>Event A500 (apiGroup 005, V01/V02)</t>
+  </si>
+  <si>
+    <t>P-10</t>
+  </si>
+  <si>
+    <t>모듈 FOTA 실패</t>
+  </si>
+  <si>
+    <t>A511 잘못된 URL / 잘못된 SHA-256</t>
+  </si>
+  <si>
+    <t>A510 102→201→900</t>
+  </si>
+  <si>
+    <t>두 경우 모두 900 errCd 9, 설치 안 함</t>
+  </si>
+  <si>
+    <t>P-11</t>
+  </si>
+  <si>
+    <t>모듈 FOTA 성공</t>
+  </si>
+  <si>
+    <t>A511 AES-256-CBC 암호화 이미지 + 올바른 SHA-256</t>
+  </si>
+  <si>
+    <t>A510 102→201→202→301, 재부팅, A100 versionChangeW true</t>
+  </si>
+  <si>
+    <t>ota_1에서 부팅, versionChangeW "true"</t>
+  </si>
+  <si>
+    <t>P-12</t>
+  </si>
+  <si>
+    <t>MCU FOTA</t>
+  </si>
+  <si>
+    <t>A521 (600바이트 이미지)</t>
+  </si>
+  <si>
+    <t>A520 102→301, MOTA_COUNT=3</t>
+  </si>
+  <si>
+    <t>MOTA_COUNT=3</t>
+  </si>
+  <si>
+    <t>P-13</t>
+  </si>
+  <si>
+    <t>MOTA 중계</t>
+  </si>
+  <si>
+    <t>MOTA_READY/DATA ×3/DATA_END=0</t>
+  </si>
+  <si>
+    <t>256/256/88 블록, MOTA_END CRC 일치, 다음 A100 versionChangeM true</t>
+  </si>
+  <si>
+    <t>CRC 2821598958 = PC 계산값, versionChangeM "true", AWS_GET 11 = CRC</t>
+  </si>
+  <si>
+    <t>P-14</t>
+  </si>
+  <si>
+    <t>인증서 갱신</t>
+  </si>
+  <si>
+    <t>클라우드 A001</t>
+  </si>
+  <si>
+    <t>AWS_RECV + /register/cert/renew 요청 + 재접속</t>
+  </si>
+  <si>
+    <t>갱신 인증서로 재접속, A100 재발행</t>
+  </si>
+  <si>
+    <t>P-15</t>
+  </si>
+  <si>
+    <t>링크 끊김</t>
+  </si>
+  <si>
+    <t>DISASSOCIATE → SMODE=99</t>
+  </si>
+  <si>
+    <t>DISCONNECT ERROR 2 → 재접속 시 CONNECT OK</t>
+  </si>
+  <si>
+    <t>일치</t>
+  </si>
+  <si>
+    <t>P-16</t>
+  </si>
+  <si>
+    <t>LWT</t>
+  </si>
+  <si>
+    <t>비정상 끊김 후 재접속 / 재부팅</t>
+  </si>
+  <si>
+    <t>브로커가 Lwt 토픽에 A102 발행</t>
+  </si>
+  <si>
+    <t>Lwt A102 수신(2회)</t>
+  </si>
+  <si>
+    <t>P-17</t>
+  </si>
+  <si>
+    <t>부팅 자동 접속</t>
+  </si>
+  <si>
+    <t>RESET=1</t>
+  </si>
+  <si>
+    <t>IP 획득 후 자동 파이프라인</t>
+  </si>
+  <si>
+    <t>CONNECT OK 0 (1회는 20초 초과로 ERROR 201 후 OK - 재현 안 됨)</t>
+  </si>
+  <si>
+    <t>P-18</t>
+  </si>
+  <si>
+    <t>설정 명령</t>
+  </si>
+  <si>
+    <t>AWS_GET/SET(null), MCU_READY, SETMIB 18/19</t>
+  </si>
+  <si>
+    <t>값 저장·조회, 잘못된 값 ERROR</t>
+  </si>
+  <si>
+    <t>P-19</t>
+  </si>
+  <si>
+    <t>앱 페어링</t>
+  </si>
+  <si>
+    <t>TCP 47000 DP0100-0400</t>
+  </si>
+  <si>
+    <t>미시험 (PC 업링크 Wi-Fi 1개)</t>
+  </si>
+  <si>
+    <t>P-20</t>
+  </si>
+  <si>
+    <t>A101 등록 해지</t>
+  </si>
+  <si>
+    <t>클라우드 A101</t>
+  </si>
+  <si>
+    <t>미시험 (AP 프로필 삭제됨)</t>
+  </si>
+  <si>
+    <t>P-21</t>
+  </si>
+  <si>
+    <t>실서버</t>
+  </si>
+  <si>
+    <t>실제 인증서버 / AWS IoT 엔드포인트</t>
+  </si>
+  <si>
+    <t>미검증 · 추후 검토 항목</t>
+  </si>
+  <si>
+    <t>대상</t>
+  </si>
+  <si>
+    <t>항목</t>
+  </si>
+  <si>
+    <t>필요 사항 / 비고</t>
+  </si>
+  <si>
+    <t>M2M</t>
+  </si>
+  <si>
+    <t>문서 본문 공백 - 사용자 별도 검토 중</t>
+  </si>
+  <si>
+    <t>파괴적 동작이라 실기 보류</t>
+  </si>
+  <si>
+    <t>폰 앱 완주 로그 미정리, PoP placeholder 교체 필요</t>
+  </si>
+  <si>
+    <t>폐기 결정(Fleet Provisioning으로 일원화), 스텁 유지</t>
+  </si>
+  <si>
+    <t>OTH</t>
   </si>
   <si>
     <t>페어링 서버 (TCP 47000)</t>
-  </si>
-  <si>
-    <t>oth_pairing.c</t>
-  </si>
-  <si>
-    <t>GEN2 프레임 DP0100-0400, AES-128 세션, SoftAP 경유만 허용. PC 업링크가 Wi-Fi 하나뿐이라 SoftAP 접속 시험 불가 - 앱/별도 단말 필요</t>
-  </si>
-  <si>
-    <t>A101 등록 해지 처리</t>
-  </si>
-  <si>
-    <t>AWS_RECV 전달 + A102 발행 + NV 전체 삭제 + 재부팅. 보드의 AP 프로필까지 지워져 시험 보류</t>
-  </si>
-  <si>
-    <t>OTH Platform 시험 기록 (2026-10-06, COM7 보드)</t>
-  </si>
-  <si>
-    <t>환경: ESP32-C3 보드(COM7), AP kangaps25, 모의 인증서버(PC 10.128.82.113:8080), MQTT broker.emqx.io(엔드포인트 대용), PC paho 클라이언트(클라우드 역할). 토픽 루트 OTHERS, MIB18=C545, MIB19=Air01</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>시험 항목</t>
-  </si>
-  <si>
-    <t>방법</t>
-  </si>
-  <si>
-    <t>기대 결과</t>
-  </si>
-  <si>
-    <t>실제 결과</t>
-  </si>
-  <si>
-    <t>P-01</t>
-  </si>
-  <si>
-    <t>인증 단계</t>
-  </si>
-  <si>
-    <t>모의 인증서버(PC LAN, http)</t>
-  </si>
-  <si>
-    <t>token 발급 → 클라이언트ID MAC_토큰, 인증서·키 발급/저장</t>
-  </si>
-  <si>
-    <t>AUTHENTICATE/CERTIFICATE/PRIVATE_KEY OK 0, AWS_GET 2 = 9CCC01C0C8E4_T0K3N7f3a</t>
-  </si>
-  <si>
-    <t>P-02</t>
-  </si>
-  <si>
-    <t>인증서 오류</t>
-  </si>
-  <si>
-    <t>공개 서비스(httpbin)로 인증서 없는 응답</t>
-  </si>
-  <si>
-    <t>CERTIFICATE ERROR 112</t>
-  </si>
-  <si>
-    <t>P-03</t>
-  </si>
-  <si>
-    <t>MQTT 접속</t>
-  </si>
-  <si>
-    <t>broker.emqx.io:8883 (TLS, 공개 CA 번들)</t>
-  </si>
-  <si>
-    <t>ROOTCA OK, CONNECT OK, Control 구독, A100 발행</t>
-  </si>
-  <si>
-    <t>A100 수신(V01=100, versionChange false)</t>
-  </si>
-  <si>
-    <t>P-04</t>
-  </si>
-  <si>
-    <t>저장 인증서 재사용</t>
-  </si>
-  <si>
-    <t>인증서버 정지 후 재부팅/재접속</t>
-  </si>
-  <si>
-    <t>서버 없이 접속</t>
-  </si>
-  <si>
-    <t>AUTHENTICATE~CONNECT OK 0</t>
-  </si>
-  <si>
-    <t>P-05</t>
-  </si>
-  <si>
-    <t>송신 봉투 / apiGroup</t>
-  </si>
-  <si>
-    <t>AWS_SEND=A110, A130</t>
-  </si>
-  <si>
-    <t>Event 토픽, apiGroup 001/003</t>
-  </si>
-  <si>
-    <t>일치, AWS_IND:SEND OK</t>
-  </si>
-  <si>
-    <t>P-06</t>
-  </si>
-  <si>
-    <t>수신 attributes</t>
-  </si>
-  <si>
-    <t>클라우드 A111 {attributes}</t>
-  </si>
-  <si>
-    <t>AWS_RECV:A111 23 {...}</t>
-  </si>
-  <si>
-    <t>AWS_RECV:A111 23 {"A03":"02","A04":"03"}</t>
-  </si>
-  <si>
-    <t>P-07</t>
-  </si>
-  <si>
-    <t>수신 평탄화</t>
-  </si>
-  <si>
-    <t>클라우드 A112 (attributes 없음)</t>
-  </si>
-  <si>
-    <t>values 필드를 JSON으로</t>
-  </si>
-  <si>
-    <t>AWS_RECV:A112 17 {"reqType":"all"}</t>
-  </si>
-  <si>
-    <t>P-08</t>
-  </si>
-  <si>
-    <t>타 장치 메시지</t>
-  </si>
-  <si>
-    <t>deviceId 다른 A111</t>
-  </si>
-  <si>
-    <t>폐기</t>
-  </si>
-  <si>
-    <t>호스트 출력 없음</t>
-  </si>
-  <si>
-    <t>P-09</t>
-  </si>
-  <si>
-    <t>버전 요청</t>
-  </si>
-  <si>
-    <t>클라우드 A502</t>
-  </si>
-  <si>
-    <t>모듈이 A500 자동 응답, 호스트 미전달</t>
-  </si>
-  <si>
-    <t>Event A500 (apiGroup 005, V01/V02)</t>
-  </si>
-  <si>
-    <t>P-10</t>
-  </si>
-  <si>
-    <t>모듈 FOTA 실패</t>
-  </si>
-  <si>
-    <t>A511 잘못된 URL / 잘못된 SHA-256</t>
-  </si>
-  <si>
-    <t>A510 102→201→900</t>
-  </si>
-  <si>
-    <t>두 경우 모두 900 errCd 9, 설치 안 함</t>
-  </si>
-  <si>
-    <t>P-11</t>
-  </si>
-  <si>
-    <t>모듈 FOTA 성공</t>
-  </si>
-  <si>
-    <t>A511 AES-256-CBC 암호화 이미지 + 올바른 SHA-256</t>
-  </si>
-  <si>
-    <t>A510 102→201→202→301, 재부팅, A100 versionChangeW true</t>
-  </si>
-  <si>
-    <t>ota_1에서 부팅, versionChangeW "true"</t>
-  </si>
-  <si>
-    <t>P-12</t>
-  </si>
-  <si>
-    <t>MCU FOTA</t>
-  </si>
-  <si>
-    <t>A521 (600바이트 이미지)</t>
-  </si>
-  <si>
-    <t>A520 102→301, MOTA_COUNT=3</t>
-  </si>
-  <si>
-    <t>MOTA_COUNT=3</t>
-  </si>
-  <si>
-    <t>P-13</t>
-  </si>
-  <si>
-    <t>MOTA 중계</t>
-  </si>
-  <si>
-    <t>MOTA_READY/DATA ×3/DATA_END=0</t>
-  </si>
-  <si>
-    <t>256/256/88 블록, MOTA_END CRC 일치, 다음 A100 versionChangeM true</t>
-  </si>
-  <si>
-    <t>CRC 2821598958 = PC 계산값, versionChangeM "true", AWS_GET 11 = CRC</t>
-  </si>
-  <si>
-    <t>P-14</t>
-  </si>
-  <si>
-    <t>인증서 갱신</t>
-  </si>
-  <si>
-    <t>클라우드 A001</t>
-  </si>
-  <si>
-    <t>AWS_RECV + /register/cert/renew 요청 + 재접속</t>
-  </si>
-  <si>
-    <t>갱신 인증서로 재접속, A100 재발행</t>
-  </si>
-  <si>
-    <t>P-15</t>
-  </si>
-  <si>
-    <t>링크 끊김</t>
-  </si>
-  <si>
-    <t>DISASSOCIATE → SMODE=99</t>
-  </si>
-  <si>
-    <t>DISCONNECT ERROR 2 → 재접속 시 CONNECT OK</t>
-  </si>
-  <si>
-    <t>일치</t>
-  </si>
-  <si>
-    <t>P-16</t>
-  </si>
-  <si>
-    <t>LWT</t>
-  </si>
-  <si>
-    <t>비정상 끊김 후 재접속 / 재부팅</t>
-  </si>
-  <si>
-    <t>브로커가 Lwt 토픽에 A102 발행</t>
-  </si>
-  <si>
-    <t>Lwt A102 수신(2회)</t>
-  </si>
-  <si>
-    <t>P-17</t>
-  </si>
-  <si>
-    <t>부팅 자동 접속</t>
-  </si>
-  <si>
-    <t>RESET=1</t>
-  </si>
-  <si>
-    <t>IP 획득 후 자동 파이프라인</t>
-  </si>
-  <si>
-    <t>CONNECT OK 0 (1회는 20초 초과로 ERROR 201 후 OK - 재현 안 됨)</t>
-  </si>
-  <si>
-    <t>P-18</t>
-  </si>
-  <si>
-    <t>설정 명령</t>
-  </si>
-  <si>
-    <t>AWS_GET/SET(null), MCU_READY, SETMIB 18/19</t>
-  </si>
-  <si>
-    <t>값 저장·조회, 잘못된 값 ERROR</t>
-  </si>
-  <si>
-    <t>P-19</t>
-  </si>
-  <si>
-    <t>앱 페어링</t>
-  </si>
-  <si>
-    <t>TCP 47000 DP0100-0400</t>
-  </si>
-  <si>
-    <t>미시험 (PC 업링크 Wi-Fi 1개)</t>
-  </si>
-  <si>
-    <t>P-20</t>
-  </si>
-  <si>
-    <t>A101 등록 해지</t>
-  </si>
-  <si>
-    <t>클라우드 A101</t>
-  </si>
-  <si>
-    <t>미시험 (AP 프로필 삭제됨)</t>
-  </si>
-  <si>
-    <t>P-21</t>
-  </si>
-  <si>
-    <t>실서버</t>
-  </si>
-  <si>
-    <t>실제 인증서버 / AWS IoT 엔드포인트</t>
-  </si>
-  <si>
-    <t>미검증 · 추후 검토 항목</t>
-  </si>
-  <si>
-    <t>대상</t>
-  </si>
-  <si>
-    <t>항목</t>
-  </si>
-  <si>
-    <t>필요 사항 / 비고</t>
-  </si>
-  <si>
-    <t>M2M</t>
-  </si>
-  <si>
-    <t>문서 본문 공백 - 사용자 별도 검토 중</t>
-  </si>
-  <si>
-    <t>파괴적 동작이라 실기 보류</t>
-  </si>
-  <si>
-    <t>폰 앱 완주 로그 미정리, PoP placeholder 교체 필요</t>
-  </si>
-  <si>
-    <t>폐기 결정(Fleet Provisioning으로 일원화), 스텁 유지</t>
-  </si>
-  <si>
-    <t>OTH</t>
   </si>
   <si>
     <t>앱 또는 별도 Wi-Fi 단말 필요</t>
@@ -2999,12 +3005,12 @@
         <v>0.9242424242424242</v>
       </c>
       <c r="D6" s="6">
-        <f>COUNTIF('OTH 명령 결과'!$D$5:$D$69,A6)</f>
-        <v>54</v>
+        <f>COUNTIF('OTH 명령 결과'!$D$5:$D$70,A6)</f>
+        <v>55</v>
       </c>
       <c r="E6" s="7">
         <f t="shared" ref="E6:E11" si="1">IF($D$12=0,0,D6/$D$12)</f>
-        <v>0.83076923076923082</v>
+        <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -3020,12 +3026,12 @@
         <v>0</v>
       </c>
       <c r="D7" s="6">
-        <f>COUNTIF('OTH 명령 결과'!$D$5:$D$69,A7)</f>
+        <f>COUNTIF('OTH 명령 결과'!$D$5:$D$70,A7)</f>
         <v>1</v>
       </c>
       <c r="E7" s="7">
         <f t="shared" si="1"/>
-        <v>1.5384615384615385E-2</v>
+        <v>1.5151515151515152E-2</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -3041,12 +3047,12 @@
         <v>3.0303030303030304E-2</v>
       </c>
       <c r="D8" s="6">
-        <f>COUNTIF('OTH 명령 결과'!$D$5:$D$69,A8)</f>
+        <f>COUNTIF('OTH 명령 결과'!$D$5:$D$70,A8)</f>
         <v>2</v>
       </c>
       <c r="E8" s="7">
         <f t="shared" si="1"/>
-        <v>3.0769230769230771E-2</v>
+        <v>3.0303030303030304E-2</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -3062,12 +3068,12 @@
         <v>1.5151515151515152E-2</v>
       </c>
       <c r="D9" s="6">
-        <f>COUNTIF('OTH 명령 결과'!$D$5:$D$69,A9)</f>
+        <f>COUNTIF('OTH 명령 결과'!$D$5:$D$70,A9)</f>
         <v>1</v>
       </c>
       <c r="E9" s="7">
         <f t="shared" si="1"/>
-        <v>1.5384615384615385E-2</v>
+        <v>1.5151515151515152E-2</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -3083,12 +3089,12 @@
         <v>0</v>
       </c>
       <c r="D10" s="6">
-        <f>COUNTIF('OTH 명령 결과'!$D$5:$D$69,A10)</f>
+        <f>COUNTIF('OTH 명령 결과'!$D$5:$D$70,A10)</f>
         <v>7</v>
       </c>
       <c r="E10" s="7">
         <f t="shared" si="1"/>
-        <v>0.1076923076923077</v>
+        <v>0.10606060606060606</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -3104,7 +3110,7 @@
         <v>3.0303030303030304E-2</v>
       </c>
       <c r="D11" s="6">
-        <f>COUNTIF('OTH 명령 결과'!$D$5:$D$69,A11)</f>
+        <f>COUNTIF('OTH 명령 결과'!$D$5:$D$70,A11)</f>
         <v>0</v>
       </c>
       <c r="E11" s="7">
@@ -3126,11 +3132,11 @@
       </c>
       <c r="D12" s="13">
         <f>SUM(D6:D11)</f>
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E12" s="14">
         <f>SUM(E6:E11)</f>
-        <v>1.0000000000000002</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
@@ -5916,7 +5922,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -7027,20 +7033,22 @@
     </row>
     <row r="60" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
       <c r="A60" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="B60" s="19" t="s">
+        <v>449</v>
+      </c>
+      <c r="C60" s="19" t="s">
         <v>581</v>
       </c>
-      <c r="B60" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="C60" s="19" t="s">
+      <c r="D60" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E60" s="19" t="s">
         <v>582</v>
       </c>
-      <c r="D60" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="E60" s="19"/>
       <c r="F60" s="19" t="s">
-        <v>227</v>
+        <v>583</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
@@ -7051,13 +7059,13 @@
         <v>449</v>
       </c>
       <c r="C61" s="19" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="D61" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E61" s="19" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="F61" s="19" t="s">
         <v>585</v>
@@ -7068,16 +7076,16 @@
         <v>177</v>
       </c>
       <c r="B62" s="19" t="s">
-        <v>70</v>
+        <v>586</v>
       </c>
       <c r="C62" s="19" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="D62" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E62" s="19" t="s">
-        <v>587</v>
+        <v>582</v>
       </c>
       <c r="F62" s="19" t="s">
         <v>588</v>
@@ -7088,7 +7096,7 @@
         <v>177</v>
       </c>
       <c r="B63" s="19" t="s">
-        <v>449</v>
+        <v>586</v>
       </c>
       <c r="C63" s="19" t="s">
         <v>589</v>
@@ -7097,7 +7105,7 @@
         <v>8</v>
       </c>
       <c r="E63" s="19" t="s">
-        <v>587</v>
+        <v>582</v>
       </c>
       <c r="F63" s="19" t="s">
         <v>590</v>
@@ -7117,50 +7125,50 @@
         <v>8</v>
       </c>
       <c r="E64" s="19" t="s">
-        <v>587</v>
+        <v>582</v>
       </c>
       <c r="F64" s="19" t="s">
         <v>592</v>
       </c>
     </row>
-    <row r="65" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="19" t="s">
         <v>177</v>
       </c>
       <c r="B65" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="C65" s="19" t="s">
         <v>593</v>
       </c>
-      <c r="C65" s="19" t="s">
+      <c r="D65" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E65" s="19" t="s">
+        <v>582</v>
+      </c>
+      <c r="F65" s="19" t="s">
         <v>594</v>
       </c>
-      <c r="D65" s="19" t="s">
-        <v>8</v>
-      </c>
-      <c r="E65" s="19" t="s">
-        <v>587</v>
-      </c>
-      <c r="F65" s="19" t="s">
-        <v>595</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="66" spans="1:6" ht="38.25" x14ac:dyDescent="0.3">
       <c r="A66" s="19" t="s">
         <v>177</v>
       </c>
       <c r="B66" s="19" t="s">
-        <v>593</v>
+        <v>70</v>
       </c>
       <c r="C66" s="19" t="s">
+        <v>595</v>
+      </c>
+      <c r="D66" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E66" s="19" t="s">
+        <v>212</v>
+      </c>
+      <c r="F66" s="19" t="s">
         <v>596</v>
-      </c>
-      <c r="D66" s="19" t="s">
-        <v>8</v>
-      </c>
-      <c r="E66" s="19" t="s">
-        <v>587</v>
-      </c>
-      <c r="F66" s="19" t="s">
-        <v>597</v>
       </c>
     </row>
     <row r="67" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
@@ -7171,19 +7179,19 @@
         <v>70</v>
       </c>
       <c r="C67" s="19" t="s">
+        <v>597</v>
+      </c>
+      <c r="D67" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E67" s="19" t="s">
+        <v>198</v>
+      </c>
+      <c r="F67" s="19" t="s">
         <v>598</v>
       </c>
-      <c r="D67" s="19" t="s">
-        <v>8</v>
-      </c>
-      <c r="E67" s="19" t="s">
-        <v>212</v>
-      </c>
-      <c r="F67" s="19" t="s">
-        <v>599</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="19" t="s">
         <v>177</v>
       </c>
@@ -7191,16 +7199,16 @@
         <v>70</v>
       </c>
       <c r="C68" s="19" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="D68" s="19" t="s">
         <v>10</v>
       </c>
       <c r="E68" s="19" t="s">
+        <v>600</v>
+      </c>
+      <c r="F68" s="19" t="s">
         <v>601</v>
-      </c>
-      <c r="F68" s="19" t="s">
-        <v>602</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
@@ -7211,22 +7219,40 @@
         <v>70</v>
       </c>
       <c r="C69" s="19" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D69" s="19" t="s">
         <v>10</v>
       </c>
       <c r="E69" s="19" t="s">
-        <v>587</v>
+        <v>582</v>
       </c>
       <c r="F69" s="19" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+      <c r="A70" s="19" t="s">
         <v>604</v>
       </c>
+      <c r="B70" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="C70" s="19" t="s">
+        <v>605</v>
+      </c>
+      <c r="D70" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E70" s="19"/>
+      <c r="F70" s="19" t="s">
+        <v>227</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F69" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <autoFilter ref="A4:F70" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <phoneticPr fontId="9" type="noConversion"/>
-  <conditionalFormatting sqref="D5:D69">
+  <conditionalFormatting sqref="D5:D70">
     <cfRule type="expression" dxfId="14" priority="1">
       <formula>$D5="검증완료"</formula>
     </cfRule>
@@ -7247,7 +7273,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="D5:D69" xr:uid="{00000000-0002-0000-0300-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D5:D70" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"검증완료,부분검증,미검증,미구현,미지원,기타"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7270,29 +7296,29 @@
   <sheetData>
     <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="F4" s="18" t="s">
         <v>17</v>
@@ -7300,19 +7326,19 @@
     </row>
     <row r="5" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
       <c r="A5" s="19" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="F5" s="19" t="s">
         <v>19</v>
@@ -7320,19 +7346,19 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="19" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="F6" s="19" t="s">
         <v>19</v>
@@ -7340,19 +7366,19 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="19" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="F7" s="19" t="s">
         <v>19</v>
@@ -7360,19 +7386,19 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="19" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="F8" s="19" t="s">
         <v>19</v>
@@ -7380,19 +7406,19 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="19" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="F9" s="19" t="s">
         <v>19</v>
@@ -7400,19 +7426,19 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="19" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="F10" s="19" t="s">
         <v>19</v>
@@ -7420,19 +7446,19 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="19" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="F11" s="19" t="s">
         <v>19</v>
@@ -7440,19 +7466,19 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="19" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="F12" s="19" t="s">
         <v>19</v>
@@ -7460,19 +7486,19 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="19" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="F13" s="19" t="s">
         <v>19</v>
@@ -7480,19 +7506,19 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="19" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="F14" s="19" t="s">
         <v>19</v>
@@ -7500,19 +7526,19 @@
     </row>
     <row r="15" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
       <c r="A15" s="19" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="F15" s="19" t="s">
         <v>19</v>
@@ -7520,19 +7546,19 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="19" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="F16" s="19" t="s">
         <v>19</v>
@@ -7540,19 +7566,19 @@
     </row>
     <row r="17" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
       <c r="A17" s="19" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="E17" s="19" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="F17" s="19" t="s">
         <v>19</v>
@@ -7560,19 +7586,19 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="19" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="F18" s="19" t="s">
         <v>19</v>
@@ -7580,19 +7606,19 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="19" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="F19" s="19" t="s">
         <v>19</v>
@@ -7600,19 +7626,19 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="19" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="E20" s="19" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="F20" s="19" t="s">
         <v>19</v>
@@ -7620,19 +7646,19 @@
     </row>
     <row r="21" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
       <c r="A21" s="19" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="F21" s="19" t="s">
         <v>20</v>
@@ -7640,19 +7666,19 @@
     </row>
     <row r="22" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
       <c r="A22" s="19" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="F22" s="19" t="s">
         <v>19</v>
@@ -7660,19 +7686,19 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="19" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="D23" s="19" t="s">
         <v>70</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="F23" s="19" t="s">
         <v>21</v>
@@ -7680,19 +7706,19 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="19" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="D24" s="19" t="s">
         <v>70</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="F24" s="19" t="s">
         <v>21</v>
@@ -7700,13 +7726,13 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="19" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="D25" s="19" t="s">
         <v>70</v>
@@ -7749,26 +7775,26 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="18" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="C3" s="18" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B4" s="19" t="s">
         <v>69</v>
@@ -7777,12 +7803,12 @@
         <v>11</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="19" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B5" s="19" t="s">
         <v>260</v>
@@ -7791,12 +7817,12 @@
         <v>10</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="19" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B6" s="19" t="s">
         <v>437</v>
@@ -7805,12 +7831,12 @@
         <v>10</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="19" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B7" s="19" t="s">
         <v>395</v>
@@ -7819,99 +7845,99 @@
         <v>13</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="19" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>600</v>
+        <v>722</v>
       </c>
       <c r="C8" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="19" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="C9" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="19" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="C10" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="19" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="C11" s="19" t="s">
         <v>9</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="19" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>9</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="25.5" x14ac:dyDescent="0.3">
       <c r="A13" s="19" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="C13" s="19" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="19" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="C14" s="19" t="s">
         <v>11</v>
@@ -7922,58 +7948,58 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="19" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="C15" s="19" t="s">
         <v>13</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="19" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="C16" s="19" t="s">
         <v>13</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="19" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="C17" s="19" t="s">
         <v>13</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="19" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="C18" s="19" t="s">
         <v>13</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Docs: Wi-Fi rejoin, start-up queue and large-message results (Phase 23)
README Phase 23 + HANDOFF: the endless rejoin and start-up command hold
queue (dd9255d) and the USB write split / MQTT reassembly (36a0a9b),
with the 2026-10-09 hardware results: AP switched off -> DISASSOCIATED,
rounds of 3 attempts with ASSOCIATED:2 every ~33 s for 6+ minutes,
rejoined by itself once the AP was back; OTH MQTT 2000/6000/8192 B
messages whole, 9000 B dropped; HTTPGET 8000 B bodies complete.
Status workbook: AUCONMODE / MQTT rows, three decisions. Comparison
workbook: rejoin and MCU relay rows (M2M now has MOTA_GET/READ/CLEAN),
M2M results 69 commands, recalculated in Excel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/doc/M2M_vs_OTH_Comparison.xlsx
+++ b/doc/M2M_vs_OTH_Comparison.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crowm\AppData\Local\Temp\claude\C--Dev-PRJ-01-ESP32-ESP32-C3\a9c7ea1d-0f66-4b51-816d-e983995d9ece\scratchpad\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\SVN\01.ESP32\OTH_ESP32_C3\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D74B6B-5DC7-4F6C-8BEF-0BA08230E09F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F8B624F-0765-453E-955D-44A792E3D711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6885" yWindow="1305" windowWidth="32475" windowHeight="18885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11460" yWindow="690" windowWidth="32475" windowHeight="18885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="요약" sheetId="1" r:id="rId1"/>
@@ -45,12 +45,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1300" uniqueCount="744">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1315" uniqueCount="754">
   <si>
     <t>M2M-AT / OTH-AT 기능 구현 비교 및 시험 결과</t>
   </si>
   <si>
-    <t>작성 2026-10-06. M2M: ESP32_C3 (GitHub M2M_ESP32_C3) / OTH: OTH_ESP32_C3 (GitHub OTH_ESP32_C, 626e615). 같은 펌웨어 소스에서 Kconfig로 명령 세트 선택</t>
+    <t>작성 2026-10-06, 갱신 2026-10-09. M2M: ESP32_C3 (GitHub M2M_ESP32_C3) / OTH: OTH_ESP32_C3 (GitHub OTH_ESP32_C, 626e615). 같은 펌웨어 소스에서 Kconfig로 명령 세트 선택</t>
   </si>
   <si>
     <t>명령 상태 집계 (각 결과 시트의 상태 열을 수식으로 집계)</t>
@@ -92,7 +92,7 @@
     <t>합계</t>
   </si>
   <si>
-    <t>※ M2M 66건(Ch.2~6 + 프로젝트 추가 명령), OTH 66행(명령 묶음 단위, AWS 볼륨은 2026-10-06 OTH Platform 결과 포함).</t>
+    <t>※ M2M 69건(Ch.2~6.7 + 프로젝트 추가 명령), OTH 66행(명령 묶음 단위, AWS 볼륨은 2026-10-06 OTH Platform 결과 포함).</t>
   </si>
   <si>
     <t>OTH Platform 시험 (2026-10-06)</t>
@@ -122,7 +122,7 @@
     <t>2. AWS: M2M은 AWS 표준 Fleet Provisioning + 임의 토픽 발행/구독(호스트 주도). OTH는 OTH Platform 전용 - SoftAP 페어링 → 인증서버 → 고정 토픽/봉투, 모듈이 자동 접속·FOTA 처리.</t>
   </si>
   <si>
-    <t>3. 펌웨어: OTH만 XMODEM(FWUPGRADE), 클라우드 암호화 FOTA, MCU 펌웨어 중계(MOTA_*) 제공.</t>
+    <t>3. 펌웨어: OTH만 XMODEM(FWUPGRADE), 클라우드 암호화 FOTA. MCU 펌웨어 중계는 양쪽(M2M MOTA_GET/READ/CLEAN pull 방식, OTH MOTA_* push 방식).</t>
   </si>
   <si>
     <t>4. 소켓: M2M net_link.c(링크 0~3) / OTH oth_sock.c(TCP 0-2, UDP 3-5, SSL 6) 별도 엔진.</t>
@@ -323,7 +323,7 @@
     <t>WF_APMODE 저장소</t>
   </si>
   <si>
-    <t>OTH는 링크 끊김 시 5초 간격 재접속</t>
+    <t>양쪽 동일 로직(공용 cmd_wifi.c): 끊김·부팅 실패 시 3회/20초 휴식 무한 재접속. 알림만 다름(M2M WF_DISCONN:DONE, OTH ASSOCIATED:2). 부팅 중 명령 보류 큐도 공용(M2M ERROR 98, OTH ERROR 7)</t>
   </si>
   <si>
     <t>IP 설정 / 상태</t>
@@ -575,7 +575,7 @@
     <t>esp-mqtt</t>
   </si>
   <si>
-    <t>M2M은 mqtts/mTLS/wss/ALPN까지 로컬 브로커 검증, OTH는 persistence 0/1/2·자동 구독</t>
+    <t>M2M은 mqtts/mTLS/wss/ALPN까지 로컬 브로커 검증, OTH는 persistence 0/1/2·자동 구독. 큰 수신 메시지: M2M 16 KB까지(초과 시 MQTT_RECV:ERROR), OTH 8 KB까지(초과 폐기)</t>
   </si>
   <si>
     <t>AWS</t>
@@ -692,10 +692,16 @@
     <t>MCU 펌웨어 중계</t>
   </si>
   <si>
+    <t>MOTA_GET, MOTA_READ, MOTA_CLEAN</t>
+  </si>
+  <si>
     <t>MOTA_START/READY/DATA/DATA_END</t>
   </si>
   <si>
-    <t>OTH만. 비활성 OTA 슬롯 사용</t>
+    <t>cmd_mota.c (M2M) / oth_fota.c (OTH)</t>
+  </si>
+  <si>
+    <t>양쪽 모두 비활성 OTA 슬롯에 저장. M2M은 MCU가 offset/len(≤4 KB)으로 당겨감(raw + CRC-32, 재요청·재개 가능), OTH는 256 B 블록 stop-and-wait 밀어주기(바이트 스터핑)</t>
   </si>
   <si>
     <t>이미지 식별 (명령체계 코드)</t>
@@ -752,7 +758,7 @@
     <t>M2M-AT 명령별 구현/시험 결과</t>
   </si>
   <si>
-    <t>출처: ESP32_C3/doc/M2M-AT_Command Set_status.xlsx (최종 갱신 2026-09-27). 상태는 이 문서 기준으로 통일(검증필요→미검증, 구현필요→미구현)</t>
+    <t>출처: ESP32_C3/doc/M2M-AT_Command Set_status.xlsx (최종 갱신 2026-10-09). 상태는 이 문서 기준으로 통일(검증필요→미검증, 구현필요→미구현)</t>
   </si>
   <si>
     <t>No</t>
@@ -1376,10 +1382,34 @@
     <t>[2026-09-27 EN 18031-1] 신규(문서 Rev 1.8). 첫 부팅 시 하드웨어 RNG 로 12자(2-9, A-Z 중 I/L/O 제외) 생성·NVS 저장, Query 로 조회(라벨/QR 인쇄용), Set 으로 8~32자 값 교체. reason 1-형식 오류, 2-프로비저닝 창 열림. COM7 실기 확인: 첫 부팅 생성, 재부팅 후 동일 값 유지, 짧은 값 거부(ERROR 1). 폰 앱으로 새 PoP 사용 세션은 미검증.</t>
   </si>
   <si>
+    <t>6.7 MCU OTA</t>
+  </si>
+  <si>
+    <t>MOTA_GET</t>
+  </si>
+  <si>
+    <t>MCU 펌웨어 이미지 다운로드(비활성 OTA 슬롯, SHA-256 선택 검증)/상태 조회</t>
+  </si>
+  <si>
+    <t>[2026-10-09 신규, 문서 Rev 1.14] tools/t_mota.py 17항목 통과, SYS_RST 후 유지, OTA_CHECK와 상호 배타 확인.</t>
+  </si>
+  <si>
+    <t>MOTA_READ</t>
+  </si>
+  <si>
+    <t>스테이징 이미지를 offset/len(≤4096 B) raw + CRC-32로 전달</t>
+  </si>
+  <si>
+    <t>MOTA_CLEAN</t>
+  </si>
+  <si>
+    <t>스테이징 이미지 폐기</t>
+  </si>
+  <si>
     <t>OTH-AT 명령별 구현/시험 결과</t>
   </si>
   <si>
-    <t>출처: OTH_ESP32_C3/doc/OTH-AT_Command_Status.xlsx (2026-10-06, AWS 볼륨은 OTH Platform 재구현 결과)</t>
+    <t>출처: OTH_ESP32_C3/doc/OTH-AT_Command_Status.xlsx (2026-10-09, AWS 볼륨은 OTH Platform 재구현 결과)</t>
   </si>
   <si>
     <t>문서</t>
@@ -1529,7 +1559,7 @@
     <t>AUCONMODE</t>
   </si>
   <si>
-    <t>mode 1: 부팅·링크 끊김 시 5초 간격 재접속. type 0-3은 저장·보고만</t>
+    <t>mode 1: 링크 끊김·부팅 접속 실패 시 무한 재접속(3초 간격 3회 → ASSOCIATED:2 → 20초 휴식 반복, DISASSOCIATED는 즉시). 같은 AP로의 재접속 명령은 연결 유지. type 0-3은 저장·보고만. 2026-10-09 AP 끔/켬 실기 확인(README Phase 23)</t>
   </si>
   <si>
     <t>SMODE</t>
@@ -1784,7 +1814,7 @@
     <t>MQTT_CONNECT / MQTT_PUB / MQTT_SUB</t>
   </si>
   <si>
-    <t>persistence 0/1/2, 자동 구독. TLS 옵션 4만(1,2 거부)</t>
+    <t>persistence 0/1/2, 자동 구독. TLS 옵션 4만(1,2 거부) / 2026-10-09: 수신 메시지 8 KB까지 재조립해 MQTT_SUB_RECV 1회로 전달(2000/6000/8192 B 실기 확인), 8 KB 초과는 알림 없이 폐기(문서에 해당 알림 없음)</t>
   </si>
   <si>
     <t>공용</t>
@@ -2276,7 +2306,7 @@
     <t>명령체계 코드 OT</t>
   </si>
   <si>
-    <t>M2M_Code Register.xlsx 명령체계코드 시트 등록 필요</t>
+    <t>2026-10-06 M2M_Code Register.xlsx에 등록 완료</t>
   </si>
 </sst>
 </file>
@@ -2960,7 +2990,7 @@
     <col min="6" max="8" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2997,12 +3027,12 @@
         <v>8</v>
       </c>
       <c r="B6" s="6">
-        <f>COUNTIF('M2M 명령 결과'!$E$5:$E$70,A6)</f>
-        <v>61</v>
+        <f>COUNTIF('M2M 명령 결과'!$E$5:$E$73,A6)</f>
+        <v>64</v>
       </c>
       <c r="C6" s="7">
         <f t="shared" ref="C6:C11" si="0">IF($B$12=0,0,B6/$B$12)</f>
-        <v>0.9242424242424242</v>
+        <v>0.92753623188405798</v>
       </c>
       <c r="D6" s="6">
         <f>COUNTIF('OTH 명령 결과'!$D$5:$D$70,A6)</f>
@@ -3018,7 +3048,7 @@
         <v>9</v>
       </c>
       <c r="B7" s="6">
-        <f>COUNTIF('M2M 명령 결과'!$E$5:$E$70,A7)</f>
+        <f>COUNTIF('M2M 명령 결과'!$E$5:$E$73,A7)</f>
         <v>0</v>
       </c>
       <c r="C7" s="7">
@@ -3039,12 +3069,12 @@
         <v>10</v>
       </c>
       <c r="B8" s="6">
-        <f>COUNTIF('M2M 명령 결과'!$E$5:$E$70,A8)</f>
+        <f>COUNTIF('M2M 명령 결과'!$E$5:$E$73,A8)</f>
         <v>2</v>
       </c>
       <c r="C8" s="7">
         <f t="shared" si="0"/>
-        <v>3.0303030303030304E-2</v>
+        <v>2.8985507246376812E-2</v>
       </c>
       <c r="D8" s="6">
         <f>COUNTIF('OTH 명령 결과'!$D$5:$D$70,A8)</f>
@@ -3060,12 +3090,12 @@
         <v>11</v>
       </c>
       <c r="B9" s="6">
-        <f>COUNTIF('M2M 명령 결과'!$E$5:$E$70,A9)</f>
+        <f>COUNTIF('M2M 명령 결과'!$E$5:$E$73,A9)</f>
         <v>1</v>
       </c>
       <c r="C9" s="7">
         <f t="shared" si="0"/>
-        <v>1.5151515151515152E-2</v>
+        <v>1.4492753623188406E-2</v>
       </c>
       <c r="D9" s="6">
         <f>COUNTIF('OTH 명령 결과'!$D$5:$D$70,A9)</f>
@@ -3081,7 +3111,7 @@
         <v>12</v>
       </c>
       <c r="B10" s="6">
-        <f>COUNTIF('M2M 명령 결과'!$E$5:$E$70,A10)</f>
+        <f>COUNTIF('M2M 명령 결과'!$E$5:$E$73,A10)</f>
         <v>0</v>
       </c>
       <c r="C10" s="7">
@@ -3102,12 +3132,12 @@
         <v>13</v>
       </c>
       <c r="B11" s="6">
-        <f>COUNTIF('M2M 명령 결과'!$E$5:$E$70,A11)</f>
+        <f>COUNTIF('M2M 명령 결과'!$E$5:$E$73,A11)</f>
         <v>2</v>
       </c>
       <c r="C11" s="7">
         <f t="shared" si="0"/>
-        <v>3.0303030303030304E-2</v>
+        <v>2.8985507246376812E-2</v>
       </c>
       <c r="D11" s="6">
         <f>COUNTIF('OTH 명령 결과'!$D$5:$D$70,A11)</f>
@@ -3124,11 +3154,11 @@
       </c>
       <c r="B12" s="13">
         <f>SUM(B6:B11)</f>
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C12" s="14">
         <f>SUM(C6:C11)</f>
-        <v>0.99999999999999989</v>
+        <v>1</v>
       </c>
       <c r="D12" s="13">
         <f>SUM(D6:D11)</f>
@@ -3299,7 +3329,7 @@
     <col min="8" max="8" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -3387,7 +3417,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="19" t="s">
         <v>37</v>
       </c>
@@ -3413,7 +3443,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="19" t="s">
         <v>37</v>
       </c>
@@ -3465,7 +3495,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="19" t="s">
         <v>37</v>
       </c>
@@ -3517,7 +3547,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="19" t="s">
         <v>73</v>
       </c>
@@ -3569,7 +3599,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="19" t="s">
         <v>73</v>
       </c>
@@ -3595,7 +3625,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="51" x14ac:dyDescent="0.3">
       <c r="A15" s="19" t="s">
         <v>73</v>
       </c>
@@ -3799,7 +3829,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="19" t="s">
         <v>124</v>
       </c>
@@ -3927,7 +3957,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="19" t="s">
         <v>144</v>
       </c>
@@ -3979,7 +4009,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="19" t="s">
         <v>144</v>
       </c>
@@ -4057,7 +4087,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="38.25" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="19" t="s">
         <v>171</v>
       </c>
@@ -4109,7 +4139,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="19" t="s">
         <v>177</v>
       </c>
@@ -4161,7 +4191,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="19" t="s">
         <v>177</v>
       </c>
@@ -4187,7 +4217,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="19" t="s">
         <v>177</v>
       </c>
@@ -4291,7 +4321,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" ht="38.25" x14ac:dyDescent="0.3">
       <c r="A42" s="19" t="s">
         <v>200</v>
       </c>
@@ -4299,19 +4329,19 @@
         <v>214</v>
       </c>
       <c r="C42" s="19" t="s">
-        <v>70</v>
+        <v>215</v>
       </c>
       <c r="D42" s="19" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E42" s="19" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="F42" s="19" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="G42" s="19" t="s">
-        <v>72</v>
+        <v>8</v>
       </c>
       <c r="H42" s="19" t="s">
         <v>8</v>
@@ -4322,19 +4352,19 @@
         <v>200</v>
       </c>
       <c r="B43" s="19" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C43" s="19" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D43" s="19" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E43" s="19" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="F43" s="19" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="G43" s="19" t="s">
         <v>8</v>
@@ -4348,19 +4378,19 @@
         <v>13</v>
       </c>
       <c r="B44" s="19" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C44" s="19" t="s">
         <v>70</v>
       </c>
       <c r="D44" s="19" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E44" s="19" t="s">
         <v>70</v>
       </c>
       <c r="F44" s="19" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G44" s="19" t="s">
         <v>72</v>
@@ -4374,19 +4404,19 @@
         <v>13</v>
       </c>
       <c r="B45" s="19" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C45" s="19" t="s">
         <v>70</v>
       </c>
       <c r="D45" s="19" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="E45" s="19" t="s">
         <v>70</v>
       </c>
       <c r="F45" s="19" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="G45" s="19" t="s">
         <v>72</v>
@@ -4395,24 +4425,24 @@
         <v>11</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="19" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B46" s="19" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C46" s="19" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D46" s="19" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E46" s="19" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="F46" s="19" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="G46" s="19" t="s">
         <v>8</v>
@@ -4453,7 +4483,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -4465,25 +4495,25 @@
     <col min="7" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="D4" s="18" t="s">
         <v>32</v>
@@ -4492,10 +4522,10 @@
         <v>3</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -4503,19 +4533,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E5" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="G5" s="19"/>
     </row>
@@ -4524,19 +4554,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="E6" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="G6" s="19"/>
     </row>
@@ -4545,42 +4575,42 @@
         <v>3</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E7" s="19" t="s">
         <v>13</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="G7" s="19" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="38.25" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="19">
         <v>4</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="E8" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="G8" s="19"/>
     </row>
@@ -4589,19 +4619,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E9" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="G9" s="19"/>
     </row>
@@ -4610,19 +4640,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="E10" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="G10" s="19"/>
     </row>
@@ -4631,40 +4661,40 @@
         <v>7</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="E11" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="G11" s="19"/>
     </row>
-    <row r="12" spans="1:7" ht="38.25" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="19">
         <v>8</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E12" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="G12" s="19"/>
     </row>
@@ -4673,40 +4703,40 @@
         <v>9</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C13" s="19" t="s">
         <v>69</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E13" s="19" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="G13" s="19"/>
     </row>
-    <row r="14" spans="1:7" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="19">
         <v>10</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E14" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="G14" s="19"/>
     </row>
@@ -4715,19 +4745,19 @@
         <v>11</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C15" s="19" t="s">
         <v>59</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="E15" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="G15" s="19"/>
     </row>
@@ -4736,40 +4766,40 @@
         <v>12</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E16" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="G16" s="19"/>
     </row>
-    <row r="17" spans="1:7" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="19">
         <v>13</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E17" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G17" s="19"/>
     </row>
@@ -4778,40 +4808,40 @@
         <v>14</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C18" s="19" t="s">
         <v>75</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="E18" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="G18" s="19"/>
     </row>
-    <row r="19" spans="1:7" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="19">
         <v>15</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C19" s="19" t="s">
         <v>89</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E19" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="G19" s="19"/>
     </row>
@@ -4820,19 +4850,19 @@
         <v>16</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C20" s="19" t="s">
         <v>80</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="E20" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G20" s="19"/>
     </row>
@@ -4841,19 +4871,19 @@
         <v>17</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E21" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="G21" s="19"/>
     </row>
@@ -4862,103 +4892,103 @@
         <v>18</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E22" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="G22" s="19"/>
     </row>
-    <row r="23" spans="1:7" ht="38.25" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="19">
         <v>19</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="E23" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="G23" s="19"/>
     </row>
-    <row r="24" spans="1:7" ht="51" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="19">
         <v>20</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="E24" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F24" s="19" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="G24" s="19"/>
     </row>
-    <row r="25" spans="1:7" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="19">
         <v>21</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C25" s="19" t="s">
         <v>94</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="E25" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F25" s="19" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="G25" s="19"/>
     </row>
-    <row r="26" spans="1:7" ht="38.25" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="19">
         <v>22</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D26" s="19" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E26" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F26" s="19" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="G26" s="19"/>
     </row>
@@ -4967,19 +4997,19 @@
         <v>23</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="C27" s="19" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E27" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F27" s="19" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="G27" s="19"/>
     </row>
@@ -4988,19 +5018,19 @@
         <v>24</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="C28" s="19" t="s">
         <v>112</v>
       </c>
       <c r="D28" s="19" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="E28" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F28" s="19" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="G28" s="19"/>
     </row>
@@ -5009,124 +5039,124 @@
         <v>25</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="D29" s="19" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E29" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F29" s="19" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="G29" s="19"/>
     </row>
-    <row r="30" spans="1:7" ht="51" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="19">
         <v>26</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C30" s="19" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="D30" s="19" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="E30" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F30" s="19" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="G30" s="19"/>
     </row>
-    <row r="31" spans="1:7" ht="38.25" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="19">
         <v>27</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D31" s="19" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="E31" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F31" s="19" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="G31" s="19"/>
     </row>
-    <row r="32" spans="1:7" ht="51" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="19">
         <v>28</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C32" s="19" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D32" s="19" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="E32" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F32" s="19" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="G32" s="19"/>
     </row>
-    <row r="33" spans="1:7" ht="51" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="19">
         <v>29</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C33" s="19" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="D33" s="19" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="E33" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F33" s="19" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="G33" s="19"/>
     </row>
-    <row r="34" spans="1:7" ht="51" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="19">
         <v>30</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C34" s="19" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="D34" s="19" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="E34" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F34" s="19" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="G34" s="19"/>
     </row>
@@ -5135,124 +5165,124 @@
         <v>31</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="D35" s="19" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E35" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F35" s="19" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G35" s="19"/>
     </row>
-    <row r="36" spans="1:7" ht="51" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="19">
         <v>32</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C36" s="19" t="s">
         <v>136</v>
       </c>
       <c r="D36" s="19" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E36" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F36" s="19" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="G36" s="19"/>
     </row>
-    <row r="37" spans="1:7" ht="51" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="19">
         <v>33</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C37" s="19" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="D37" s="19" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="E37" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F37" s="19" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="G37" s="19"/>
     </row>
-    <row r="38" spans="1:7" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="19">
         <v>34</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C38" s="19" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="D38" s="19" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="E38" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F38" s="19" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="G38" s="19"/>
     </row>
-    <row r="39" spans="1:7" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="19">
         <v>35</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C39" s="19" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D39" s="19" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="E39" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F39" s="19" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="G39" s="19"/>
     </row>
-    <row r="40" spans="1:7" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="19">
         <v>36</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C40" s="19" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="D40" s="19" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="E40" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F40" s="19" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="G40" s="19"/>
     </row>
@@ -5261,40 +5291,40 @@
         <v>37</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C41" s="19" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="D41" s="19" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="E41" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F41" s="19" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="G41" s="19"/>
     </row>
-    <row r="42" spans="1:7" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="19">
         <v>38</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C42" s="19" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D42" s="19" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="E42" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F42" s="19" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="G42" s="19"/>
     </row>
@@ -5303,19 +5333,19 @@
         <v>39</v>
       </c>
       <c r="B43" s="19" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C43" s="19" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="D43" s="19" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="E43" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F43" s="19" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="G43" s="19"/>
     </row>
@@ -5324,19 +5354,19 @@
         <v>40</v>
       </c>
       <c r="B44" s="19" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C44" s="19" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="D44" s="19" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="E44" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F44" s="19" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="G44" s="19"/>
     </row>
@@ -5345,103 +5375,103 @@
         <v>41</v>
       </c>
       <c r="B45" s="19" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C45" s="19" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="D45" s="19" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="E45" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F45" s="19" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="G45" s="19"/>
     </row>
-    <row r="46" spans="1:7" ht="38.25" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="19">
         <v>42</v>
       </c>
       <c r="B46" s="19" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C46" s="19" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="D46" s="19" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="E46" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F46" s="19" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="G46" s="19"/>
     </row>
-    <row r="47" spans="1:7" ht="38.25" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="19">
         <v>43</v>
       </c>
       <c r="B47" s="19" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="C47" s="19" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="D47" s="19" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="E47" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F47" s="19" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="G47" s="19"/>
     </row>
-    <row r="48" spans="1:7" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="19">
         <v>44</v>
       </c>
       <c r="B48" s="19" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="C48" s="19" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="D48" s="19" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E48" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F48" s="19" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="G48" s="19"/>
     </row>
-    <row r="49" spans="1:7" ht="38.25" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="19">
         <v>45</v>
       </c>
       <c r="B49" s="19" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="C49" s="19" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="D49" s="19" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="E49" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F49" s="19" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="G49" s="19"/>
     </row>
@@ -5450,61 +5480,61 @@
         <v>46</v>
       </c>
       <c r="B50" s="19" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="C50" s="19" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="D50" s="19" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="E50" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F50" s="19" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="G50" s="19"/>
     </row>
-    <row r="51" spans="1:7" ht="51" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="19">
         <v>47</v>
       </c>
       <c r="B51" s="19" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="C51" s="19" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="D51" s="19" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="E51" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F51" s="19" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="G51" s="19"/>
     </row>
-    <row r="52" spans="1:7" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="19">
         <v>48</v>
       </c>
       <c r="B52" s="19" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="C52" s="19" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="D52" s="19" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="E52" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F52" s="19" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="G52" s="19"/>
     </row>
@@ -5513,19 +5543,19 @@
         <v>49</v>
       </c>
       <c r="B53" s="19" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="C53" s="19" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="D53" s="19" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="E53" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F53" s="19" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="G53" s="19"/>
     </row>
@@ -5534,19 +5564,19 @@
         <v>50</v>
       </c>
       <c r="B54" s="19" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="C54" s="19" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="D54" s="19" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="E54" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F54" s="19" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="G54" s="19"/>
     </row>
@@ -5555,126 +5585,126 @@
         <v>51</v>
       </c>
       <c r="B55" s="19" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="C55" s="19" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="D55" s="19" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="E55" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F55" s="19" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="G55" s="19"/>
     </row>
-    <row r="56" spans="1:7" ht="38.25" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="19">
         <v>52</v>
       </c>
       <c r="B56" s="19" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="C56" s="19" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="D56" s="19" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="E56" s="19" t="s">
         <v>13</v>
       </c>
       <c r="F56" s="19" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="G56" s="19" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" ht="38.25" x14ac:dyDescent="0.3">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="19">
         <v>53</v>
       </c>
       <c r="B57" s="19" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="C57" s="19" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="D57" s="19" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="E57" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F57" s="19" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="G57" s="19"/>
     </row>
-    <row r="58" spans="1:7" ht="51" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="19">
         <v>54</v>
       </c>
       <c r="B58" s="19" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="C58" s="19" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D58" s="19" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="E58" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F58" s="19" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="G58" s="19"/>
     </row>
-    <row r="59" spans="1:7" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="19">
         <v>55</v>
       </c>
       <c r="B59" s="19" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="C59" s="19" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="D59" s="19" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="E59" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F59" s="19" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="G59" s="19"/>
     </row>
-    <row r="60" spans="1:7" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="19">
         <v>56</v>
       </c>
       <c r="B60" s="19" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="C60" s="19" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="D60" s="19" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="E60" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F60" s="19" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="G60" s="19"/>
     </row>
@@ -5683,19 +5713,19 @@
         <v>57</v>
       </c>
       <c r="B61" s="19" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="C61" s="19" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="D61" s="19" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="E61" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F61" s="19" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="G61" s="19"/>
     </row>
@@ -5704,40 +5734,40 @@
         <v>58</v>
       </c>
       <c r="B62" s="19" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="C62" s="19" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="D62" s="19" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="E62" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F62" s="19" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="G62" s="19"/>
     </row>
-    <row r="63" spans="1:7" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="19">
         <v>59</v>
       </c>
       <c r="B63" s="19" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="C63" s="19" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="D63" s="19" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="E63" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F63" s="19" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="G63" s="19"/>
     </row>
@@ -5746,19 +5776,19 @@
         <v>60</v>
       </c>
       <c r="B64" s="19" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="C64" s="19" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D64" s="19" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="E64" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F64" s="19" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="G64" s="19"/>
     </row>
@@ -5767,126 +5797,189 @@
         <v>61</v>
       </c>
       <c r="B65" s="19" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="C65" s="19" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D65" s="19" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="E65" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F65" s="19" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="G65" s="19"/>
     </row>
-    <row r="66" spans="1:7" ht="38.25" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="19">
         <v>62</v>
       </c>
       <c r="B66" s="19" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C66" s="19" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="D66" s="19" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E66" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F66" s="19" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="G66" s="19"/>
     </row>
-    <row r="67" spans="1:7" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="19">
         <v>63</v>
       </c>
       <c r="B67" s="19" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C67" s="19" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="D67" s="19" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="E67" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F67" s="19" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="G67" s="19"/>
     </row>
-    <row r="68" spans="1:7" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="19">
         <v>64</v>
       </c>
       <c r="B68" s="19" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="C68" s="19" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="D68" s="19" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="E68" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F68" s="19" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="G68" s="19"/>
     </row>
-    <row r="69" spans="1:7" ht="38.25" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="19">
         <v>65</v>
       </c>
       <c r="B69" s="19" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="C69" s="19" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="D69" s="19" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="E69" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F69" s="19" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="G69" s="19"/>
     </row>
-    <row r="70" spans="1:7" ht="38.25" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="19">
         <v>66</v>
       </c>
       <c r="B70" s="19" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="C70" s="19" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="D70" s="19" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="E70" s="19" t="s">
         <v>8</v>
       </c>
       <c r="F70" s="19" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="G70" s="19"/>
+    </row>
+    <row r="71" spans="1:7" ht="25.5" x14ac:dyDescent="0.3">
+      <c r="A71" s="19">
+        <v>67</v>
+      </c>
+      <c r="B71" s="19" t="s">
+        <v>445</v>
+      </c>
+      <c r="C71" s="19" t="s">
+        <v>446</v>
+      </c>
+      <c r="D71" s="19" t="s">
+        <v>447</v>
+      </c>
+      <c r="E71" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="F71" s="19" t="s">
+        <v>448</v>
+      </c>
+      <c r="G71" s="19"/>
+    </row>
+    <row r="72" spans="1:7" ht="25.5" x14ac:dyDescent="0.3">
+      <c r="A72" s="19">
+        <v>68</v>
+      </c>
+      <c r="B72" s="19" t="s">
+        <v>445</v>
+      </c>
+      <c r="C72" s="19" t="s">
+        <v>449</v>
+      </c>
+      <c r="D72" s="19" t="s">
+        <v>450</v>
+      </c>
+      <c r="E72" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="F72" s="19" t="s">
+        <v>448</v>
+      </c>
+      <c r="G72" s="19"/>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A73" s="19">
+        <v>69</v>
+      </c>
+      <c r="B73" s="19" t="s">
+        <v>445</v>
+      </c>
+      <c r="C73" s="19" t="s">
+        <v>451</v>
+      </c>
+      <c r="D73" s="19" t="s">
+        <v>452</v>
+      </c>
+      <c r="E73" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="F73" s="19" t="s">
+        <v>448</v>
+      </c>
+      <c r="G73" s="19"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:G70" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
@@ -5933,63 +6026,63 @@
     <col min="6" max="6" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>443</v>
+        <v>453</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>444</v>
+        <v>454</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="s">
-        <v>445</v>
+        <v>455</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>446</v>
+        <v>456</v>
       </c>
       <c r="D4" s="18" t="s">
         <v>3</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>447</v>
+        <v>457</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>450</v>
+        <v>460</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>451</v>
+        <v>461</v>
       </c>
       <c r="F5" s="19"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>452</v>
+        <v>462</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>8</v>
@@ -5998,251 +6091,251 @@
         <v>45</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>453</v>
+        <v>463</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>454</v>
+        <v>464</v>
       </c>
       <c r="D7" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F7" s="19"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>455</v>
+        <v>465</v>
       </c>
       <c r="D8" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>456</v>
+        <v>466</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>458</v>
+        <v>468</v>
       </c>
       <c r="D9" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>459</v>
+        <v>469</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>460</v>
+        <v>470</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>461</v>
+        <v>471</v>
       </c>
       <c r="D10" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>462</v>
+        <v>472</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>464</v>
+        <v>474</v>
       </c>
       <c r="D11" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>465</v>
+        <v>475</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>466</v>
+        <v>476</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>467</v>
+        <v>477</v>
       </c>
       <c r="D12" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>468</v>
+        <v>478</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>469</v>
+        <v>479</v>
       </c>
       <c r="D13" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>470</v>
+        <v>480</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>471</v>
+        <v>481</v>
       </c>
       <c r="D14" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>472</v>
+        <v>482</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>473</v>
+        <v>483</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>474</v>
+        <v>484</v>
       </c>
       <c r="D15" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>475</v>
+        <v>485</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>476</v>
+        <v>486</v>
       </c>
       <c r="D16" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>477</v>
+        <v>487</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>478</v>
+        <v>488</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D17" s="19" t="s">
         <v>12</v>
       </c>
       <c r="E17" s="19"/>
       <c r="F17" s="19" t="s">
-        <v>479</v>
+        <v>489</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>481</v>
+        <v>491</v>
       </c>
       <c r="D18" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>482</v>
+        <v>492</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>483</v>
+        <v>493</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
       <c r="C19" s="19" t="s">
         <v>81</v>
@@ -6251,21 +6344,21 @@
         <v>8</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>484</v>
+        <v>494</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>485</v>
+        <v>495</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>486</v>
+        <v>496</v>
       </c>
       <c r="D20" s="19" t="s">
         <v>8</v>
@@ -6274,54 +6367,54 @@
         <v>86</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>487</v>
+        <v>497</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>488</v>
+        <v>498</v>
       </c>
       <c r="D21" s="19" t="s">
         <v>12</v>
       </c>
       <c r="E21" s="19"/>
       <c r="F21" s="19" t="s">
-        <v>489</v>
+        <v>499</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>490</v>
+        <v>500</v>
       </c>
       <c r="D22" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="F22" s="19"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>491</v>
+        <v>501</v>
       </c>
       <c r="D23" s="19" t="s">
         <v>8</v>
@@ -6330,18 +6423,18 @@
         <v>86</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
       <c r="A24" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>493</v>
+        <v>503</v>
       </c>
       <c r="D24" s="19" t="s">
         <v>8</v>
@@ -6350,78 +6443,78 @@
         <v>91</v>
       </c>
       <c r="F24" s="19" t="s">
-        <v>494</v>
+        <v>504</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>495</v>
+        <v>505</v>
       </c>
       <c r="D25" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E25" s="19" t="s">
-        <v>496</v>
+        <v>506</v>
       </c>
       <c r="F25" s="19" t="s">
-        <v>497</v>
+        <v>507</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>498</v>
+        <v>508</v>
       </c>
       <c r="D26" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>499</v>
+        <v>509</v>
       </c>
       <c r="F26" s="19" t="s">
-        <v>500</v>
+        <v>510</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
       <c r="C27" s="19" t="s">
-        <v>501</v>
+        <v>511</v>
       </c>
       <c r="D27" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E27" s="19" t="s">
-        <v>502</v>
+        <v>512</v>
       </c>
       <c r="F27" s="19" t="s">
-        <v>503</v>
+        <v>513</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>504</v>
+        <v>514</v>
       </c>
       <c r="C28" s="19" t="s">
-        <v>505</v>
+        <v>515</v>
       </c>
       <c r="D28" s="19" t="s">
         <v>8</v>
@@ -6430,18 +6523,18 @@
         <v>105</v>
       </c>
       <c r="F28" s="19" t="s">
-        <v>506</v>
+        <v>516</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>504</v>
+        <v>514</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>507</v>
+        <v>517</v>
       </c>
       <c r="D29" s="19" t="s">
         <v>8</v>
@@ -6450,18 +6543,18 @@
         <v>110</v>
       </c>
       <c r="F29" s="19" t="s">
-        <v>508</v>
+        <v>518</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>504</v>
+        <v>514</v>
       </c>
       <c r="C30" s="19" t="s">
-        <v>509</v>
+        <v>519</v>
       </c>
       <c r="D30" s="19" t="s">
         <v>8</v>
@@ -6471,15 +6564,15 @@
       </c>
       <c r="F30" s="19"/>
     </row>
-    <row r="31" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>510</v>
+        <v>520</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>511</v>
+        <v>521</v>
       </c>
       <c r="D31" s="19" t="s">
         <v>8</v>
@@ -6488,72 +6581,72 @@
         <v>114</v>
       </c>
       <c r="F31" s="19" t="s">
-        <v>512</v>
+        <v>522</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>510</v>
+        <v>520</v>
       </c>
       <c r="C32" s="19" t="s">
-        <v>513</v>
+        <v>523</v>
       </c>
       <c r="D32" s="19" t="s">
         <v>12</v>
       </c>
       <c r="E32" s="19"/>
       <c r="F32" s="19" t="s">
-        <v>514</v>
+        <v>524</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>510</v>
+        <v>520</v>
       </c>
       <c r="C33" s="19" t="s">
-        <v>515</v>
+        <v>525</v>
       </c>
       <c r="D33" s="19" t="s">
         <v>12</v>
       </c>
       <c r="E33" s="19"/>
       <c r="F33" s="19" t="s">
-        <v>516</v>
+        <v>526</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>510</v>
+        <v>520</v>
       </c>
       <c r="C34" s="19" t="s">
-        <v>517</v>
+        <v>527</v>
       </c>
       <c r="D34" s="19" t="s">
         <v>12</v>
       </c>
       <c r="E34" s="19"/>
       <c r="F34" s="19" t="s">
-        <v>518</v>
+        <v>528</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>519</v>
+        <v>529</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>520</v>
+        <v>530</v>
       </c>
       <c r="D35" s="19" t="s">
         <v>8</v>
@@ -6565,189 +6658,189 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>519</v>
+        <v>529</v>
       </c>
       <c r="C36" s="19" t="s">
-        <v>521</v>
+        <v>531</v>
       </c>
       <c r="D36" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E36" s="19" t="s">
-        <v>522</v>
+        <v>532</v>
       </c>
       <c r="F36" s="19" t="s">
-        <v>523</v>
+        <v>533</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>519</v>
+        <v>529</v>
       </c>
       <c r="C37" s="19" t="s">
-        <v>524</v>
+        <v>534</v>
       </c>
       <c r="D37" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E37" s="19" t="s">
-        <v>522</v>
+        <v>532</v>
       </c>
       <c r="F37" s="19" t="s">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>519</v>
+        <v>529</v>
       </c>
       <c r="C38" s="19" t="s">
-        <v>526</v>
+        <v>536</v>
       </c>
       <c r="D38" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E38" s="19" t="s">
-        <v>522</v>
+        <v>532</v>
       </c>
       <c r="F38" s="19" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>519</v>
+        <v>529</v>
       </c>
       <c r="C39" s="19" t="s">
-        <v>528</v>
+        <v>538</v>
       </c>
       <c r="D39" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E39" s="19" t="s">
-        <v>522</v>
+        <v>532</v>
       </c>
       <c r="F39" s="19" t="s">
-        <v>529</v>
+        <v>539</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>519</v>
+        <v>529</v>
       </c>
       <c r="C40" s="19" t="s">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="D40" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E40" s="19" t="s">
-        <v>531</v>
+        <v>541</v>
       </c>
       <c r="F40" s="19" t="s">
-        <v>532</v>
+        <v>542</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>519</v>
+        <v>529</v>
       </c>
       <c r="C41" s="19" t="s">
-        <v>533</v>
+        <v>543</v>
       </c>
       <c r="D41" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E41" s="19" t="s">
-        <v>522</v>
+        <v>532</v>
       </c>
       <c r="F41" s="19"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>519</v>
+        <v>529</v>
       </c>
       <c r="C42" s="19" t="s">
-        <v>534</v>
+        <v>544</v>
       </c>
       <c r="D42" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E42" s="19" t="s">
-        <v>535</v>
+        <v>545</v>
       </c>
       <c r="F42" s="19" t="s">
-        <v>536</v>
+        <v>546</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B43" s="19" t="s">
-        <v>519</v>
+        <v>529</v>
       </c>
       <c r="C43" s="19" t="s">
-        <v>537</v>
+        <v>547</v>
       </c>
       <c r="D43" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E43" s="19" t="s">
-        <v>538</v>
+        <v>548</v>
       </c>
       <c r="F43" s="19"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B44" s="19" t="s">
-        <v>519</v>
+        <v>529</v>
       </c>
       <c r="C44" s="19" t="s">
-        <v>539</v>
+        <v>549</v>
       </c>
       <c r="D44" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E44" s="19" t="s">
-        <v>540</v>
+        <v>550</v>
       </c>
       <c r="F44" s="19" t="s">
-        <v>541</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B45" s="19" t="s">
-        <v>542</v>
+        <v>552</v>
       </c>
       <c r="C45" s="19" t="s">
-        <v>543</v>
+        <v>553</v>
       </c>
       <c r="D45" s="19" t="s">
         <v>8</v>
@@ -6756,136 +6849,136 @@
         <v>133</v>
       </c>
       <c r="F45" s="19" t="s">
-        <v>544</v>
+        <v>554</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B46" s="19" t="s">
-        <v>542</v>
+        <v>552</v>
       </c>
       <c r="C46" s="19" t="s">
-        <v>545</v>
+        <v>555</v>
       </c>
       <c r="D46" s="19" t="s">
         <v>9</v>
       </c>
       <c r="E46" s="19" t="s">
-        <v>546</v>
+        <v>556</v>
       </c>
       <c r="F46" s="19" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B47" s="19" t="s">
-        <v>548</v>
+        <v>558</v>
       </c>
       <c r="C47" s="19" t="s">
-        <v>549</v>
+        <v>559</v>
       </c>
       <c r="D47" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E47" s="19" t="s">
-        <v>550</v>
+        <v>560</v>
       </c>
       <c r="F47" s="19" t="s">
-        <v>551</v>
+        <v>561</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B48" s="19" t="s">
-        <v>548</v>
+        <v>558</v>
       </c>
       <c r="C48" s="19" t="s">
-        <v>552</v>
+        <v>562</v>
       </c>
       <c r="D48" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E48" s="19" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="F48" s="19" t="s">
-        <v>553</v>
+        <v>563</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B49" s="19" t="s">
-        <v>554</v>
+        <v>564</v>
       </c>
       <c r="C49" s="19" t="s">
-        <v>555</v>
+        <v>565</v>
       </c>
       <c r="D49" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E49" s="19" t="s">
-        <v>556</v>
+        <v>566</v>
       </c>
       <c r="F49" s="19" t="s">
-        <v>557</v>
+        <v>567</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B50" s="19" t="s">
-        <v>554</v>
+        <v>564</v>
       </c>
       <c r="C50" s="19" t="s">
-        <v>558</v>
+        <v>568</v>
       </c>
       <c r="D50" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E50" s="19" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="F50" s="19" t="s">
-        <v>559</v>
+        <v>569</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B51" s="19" t="s">
-        <v>560</v>
+        <v>570</v>
       </c>
       <c r="C51" s="19" t="s">
-        <v>561</v>
+        <v>571</v>
       </c>
       <c r="D51" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E51" s="19" t="s">
-        <v>562</v>
+        <v>572</v>
       </c>
       <c r="F51" s="19"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B52" s="19" t="s">
-        <v>560</v>
+        <v>570</v>
       </c>
       <c r="C52" s="19" t="s">
-        <v>563</v>
+        <v>573</v>
       </c>
       <c r="D52" s="19" t="s">
         <v>8</v>
@@ -6894,63 +6987,63 @@
         <v>166</v>
       </c>
       <c r="F52" s="19" t="s">
-        <v>564</v>
+        <v>574</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B53" s="19" t="s">
-        <v>560</v>
+        <v>570</v>
       </c>
       <c r="C53" s="19" t="s">
-        <v>565</v>
+        <v>575</v>
       </c>
       <c r="D53" s="19" t="s">
         <v>12</v>
       </c>
       <c r="E53" s="19"/>
       <c r="F53" s="19" t="s">
-        <v>566</v>
+        <v>576</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B54" s="19" t="s">
-        <v>567</v>
+        <v>577</v>
       </c>
       <c r="C54" s="19" t="s">
-        <v>568</v>
+        <v>578</v>
       </c>
       <c r="D54" s="19" t="s">
         <v>12</v>
       </c>
       <c r="E54" s="19"/>
       <c r="F54" s="19" t="s">
-        <v>566</v>
+        <v>576</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="19" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B55" s="19" t="s">
-        <v>569</v>
+        <v>579</v>
       </c>
       <c r="C55" s="19" t="s">
-        <v>570</v>
+        <v>580</v>
       </c>
       <c r="D55" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E55" s="19" t="s">
-        <v>571</v>
+        <v>581</v>
       </c>
       <c r="F55" s="19" t="s">
-        <v>572</v>
+        <v>582</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
@@ -6958,19 +7051,19 @@
         <v>171</v>
       </c>
       <c r="B56" s="19" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="C56" s="19" t="s">
-        <v>573</v>
+        <v>583</v>
       </c>
       <c r="D56" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E56" s="19" t="s">
-        <v>574</v>
+        <v>584</v>
       </c>
       <c r="F56" s="19" t="s">
-        <v>575</v>
+        <v>585</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
@@ -6978,30 +7071,30 @@
         <v>171</v>
       </c>
       <c r="B57" s="19" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="C57" s="19" t="s">
-        <v>576</v>
+        <v>586</v>
       </c>
       <c r="D57" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E57" s="19" t="s">
-        <v>574</v>
+        <v>584</v>
       </c>
       <c r="F57" s="19" t="s">
-        <v>577</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="19" t="s">
         <v>171</v>
       </c>
       <c r="B58" s="19" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="C58" s="19" t="s">
-        <v>578</v>
+        <v>588</v>
       </c>
       <c r="D58" s="19" t="s">
         <v>8</v>
@@ -7010,7 +7103,7 @@
         <v>175</v>
       </c>
       <c r="F58" s="19" t="s">
-        <v>579</v>
+        <v>589</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
@@ -7018,57 +7111,57 @@
         <v>171</v>
       </c>
       <c r="B59" s="19" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="C59" s="19" t="s">
-        <v>552</v>
+        <v>562</v>
       </c>
       <c r="D59" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E59" s="19" t="s">
-        <v>580</v>
+        <v>590</v>
       </c>
       <c r="F59" s="19"/>
     </row>
-    <row r="60" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="19" t="s">
         <v>177</v>
       </c>
       <c r="B60" s="19" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="C60" s="19" t="s">
-        <v>581</v>
+        <v>591</v>
       </c>
       <c r="D60" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E60" s="19" t="s">
-        <v>582</v>
+        <v>592</v>
       </c>
       <c r="F60" s="19" t="s">
-        <v>583</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="19" t="s">
         <v>177</v>
       </c>
       <c r="B61" s="19" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="C61" s="19" t="s">
-        <v>584</v>
+        <v>594</v>
       </c>
       <c r="D61" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E61" s="19" t="s">
-        <v>582</v>
+        <v>592</v>
       </c>
       <c r="F61" s="19" t="s">
-        <v>585</v>
+        <v>595</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
@@ -7076,39 +7169,39 @@
         <v>177</v>
       </c>
       <c r="B62" s="19" t="s">
-        <v>586</v>
+        <v>596</v>
       </c>
       <c r="C62" s="19" t="s">
-        <v>587</v>
+        <v>597</v>
       </c>
       <c r="D62" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E62" s="19" t="s">
-        <v>582</v>
+        <v>592</v>
       </c>
       <c r="F62" s="19" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="19" t="s">
         <v>177</v>
       </c>
       <c r="B63" s="19" t="s">
-        <v>586</v>
+        <v>596</v>
       </c>
       <c r="C63" s="19" t="s">
-        <v>589</v>
+        <v>599</v>
       </c>
       <c r="D63" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E63" s="19" t="s">
-        <v>582</v>
+        <v>592</v>
       </c>
       <c r="F63" s="19" t="s">
-        <v>590</v>
+        <v>600</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
@@ -7119,16 +7212,16 @@
         <v>70</v>
       </c>
       <c r="C64" s="19" t="s">
-        <v>591</v>
+        <v>601</v>
       </c>
       <c r="D64" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E64" s="19" t="s">
-        <v>582</v>
+        <v>592</v>
       </c>
       <c r="F64" s="19" t="s">
-        <v>592</v>
+        <v>602</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
@@ -7139,19 +7232,19 @@
         <v>70</v>
       </c>
       <c r="C65" s="19" t="s">
-        <v>593</v>
+        <v>603</v>
       </c>
       <c r="D65" s="19" t="s">
         <v>8</v>
       </c>
       <c r="E65" s="19" t="s">
-        <v>582</v>
+        <v>592</v>
       </c>
       <c r="F65" s="19" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" ht="38.25" x14ac:dyDescent="0.3">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="19" t="s">
         <v>177</v>
       </c>
@@ -7159,7 +7252,7 @@
         <v>70</v>
       </c>
       <c r="C66" s="19" t="s">
-        <v>595</v>
+        <v>605</v>
       </c>
       <c r="D66" s="19" t="s">
         <v>8</v>
@@ -7168,10 +7261,10 @@
         <v>212</v>
       </c>
       <c r="F66" s="19" t="s">
-        <v>596</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="19" t="s">
         <v>177</v>
       </c>
@@ -7179,7 +7272,7 @@
         <v>70</v>
       </c>
       <c r="C67" s="19" t="s">
-        <v>597</v>
+        <v>607</v>
       </c>
       <c r="D67" s="19" t="s">
         <v>8</v>
@@ -7188,7 +7281,7 @@
         <v>198</v>
       </c>
       <c r="F67" s="19" t="s">
-        <v>598</v>
+        <v>608</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
@@ -7199,16 +7292,16 @@
         <v>70</v>
       </c>
       <c r="C68" s="19" t="s">
-        <v>599</v>
+        <v>609</v>
       </c>
       <c r="D68" s="19" t="s">
         <v>10</v>
       </c>
       <c r="E68" s="19" t="s">
-        <v>600</v>
+        <v>610</v>
       </c>
       <c r="F68" s="19" t="s">
-        <v>601</v>
+        <v>611</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
@@ -7219,34 +7312,34 @@
         <v>70</v>
       </c>
       <c r="C69" s="19" t="s">
-        <v>602</v>
+        <v>612</v>
       </c>
       <c r="D69" s="19" t="s">
         <v>10</v>
       </c>
       <c r="E69" s="19" t="s">
-        <v>582</v>
+        <v>592</v>
       </c>
       <c r="F69" s="19" t="s">
-        <v>603</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="19" t="s">
-        <v>604</v>
+        <v>614</v>
       </c>
       <c r="B70" s="19" t="s">
         <v>70</v>
       </c>
       <c r="C70" s="19" t="s">
-        <v>605</v>
+        <v>615</v>
       </c>
       <c r="D70" s="19" t="s">
         <v>11</v>
       </c>
       <c r="E70" s="19"/>
       <c r="F70" s="19" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -7294,51 +7387,51 @@
     <col min="6" max="6" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>606</v>
+        <v>616</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>607</v>
+        <v>617</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="s">
-        <v>608</v>
+        <v>618</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>609</v>
+        <v>619</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>610</v>
+        <v>620</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>611</v>
+        <v>621</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>612</v>
+        <v>622</v>
       </c>
       <c r="F4" s="18" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="19" t="s">
-        <v>613</v>
+        <v>623</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>614</v>
+        <v>624</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>615</v>
+        <v>625</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>616</v>
+        <v>626</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>617</v>
+        <v>627</v>
       </c>
       <c r="F5" s="19" t="s">
         <v>19</v>
@@ -7346,19 +7439,19 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="19" t="s">
-        <v>618</v>
+        <v>628</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>619</v>
+        <v>629</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>620</v>
+        <v>630</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>621</v>
+        <v>631</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>621</v>
+        <v>631</v>
       </c>
       <c r="F6" s="19" t="s">
         <v>19</v>
@@ -7366,19 +7459,19 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="19" t="s">
-        <v>622</v>
+        <v>632</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>623</v>
+        <v>633</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>624</v>
+        <v>634</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>625</v>
+        <v>635</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>626</v>
+        <v>636</v>
       </c>
       <c r="F7" s="19" t="s">
         <v>19</v>
@@ -7386,19 +7479,19 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="19" t="s">
-        <v>627</v>
+        <v>637</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>628</v>
+        <v>638</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>629</v>
+        <v>639</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>630</v>
+        <v>640</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>631</v>
+        <v>641</v>
       </c>
       <c r="F8" s="19" t="s">
         <v>19</v>
@@ -7406,19 +7499,19 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="19" t="s">
-        <v>632</v>
+        <v>642</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>633</v>
+        <v>643</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>634</v>
+        <v>644</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>635</v>
+        <v>645</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>636</v>
+        <v>646</v>
       </c>
       <c r="F9" s="19" t="s">
         <v>19</v>
@@ -7426,19 +7519,19 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="19" t="s">
-        <v>637</v>
+        <v>647</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>638</v>
+        <v>648</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>639</v>
+        <v>649</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>640</v>
+        <v>650</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>641</v>
+        <v>651</v>
       </c>
       <c r="F10" s="19" t="s">
         <v>19</v>
@@ -7446,19 +7539,19 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="19" t="s">
-        <v>642</v>
+        <v>652</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>643</v>
+        <v>653</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>644</v>
+        <v>654</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>645</v>
+        <v>655</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>646</v>
+        <v>656</v>
       </c>
       <c r="F11" s="19" t="s">
         <v>19</v>
@@ -7466,19 +7559,19 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="19" t="s">
-        <v>647</v>
+        <v>657</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>648</v>
+        <v>658</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>649</v>
+        <v>659</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>650</v>
+        <v>660</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>651</v>
+        <v>661</v>
       </c>
       <c r="F12" s="19" t="s">
         <v>19</v>
@@ -7486,19 +7579,19 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="19" t="s">
-        <v>652</v>
+        <v>662</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>653</v>
+        <v>663</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>654</v>
+        <v>664</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>655</v>
+        <v>665</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>656</v>
+        <v>666</v>
       </c>
       <c r="F13" s="19" t="s">
         <v>19</v>
@@ -7506,39 +7599,39 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="19" t="s">
-        <v>657</v>
+        <v>667</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>658</v>
+        <v>668</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>659</v>
+        <v>669</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>660</v>
+        <v>670</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>661</v>
+        <v>671</v>
       </c>
       <c r="F14" s="19" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="19" t="s">
-        <v>662</v>
+        <v>672</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>663</v>
+        <v>673</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>664</v>
+        <v>674</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>665</v>
+        <v>675</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>666</v>
+        <v>676</v>
       </c>
       <c r="F15" s="19" t="s">
         <v>19</v>
@@ -7546,39 +7639,39 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="19" t="s">
-        <v>667</v>
+        <v>677</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>668</v>
+        <v>678</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>669</v>
+        <v>679</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>670</v>
+        <v>680</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>671</v>
+        <v>681</v>
       </c>
       <c r="F16" s="19" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="19" t="s">
-        <v>672</v>
+        <v>682</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>673</v>
+        <v>683</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>674</v>
+        <v>684</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>675</v>
+        <v>685</v>
       </c>
       <c r="E17" s="19" t="s">
-        <v>676</v>
+        <v>686</v>
       </c>
       <c r="F17" s="19" t="s">
         <v>19</v>
@@ -7586,19 +7679,19 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="19" t="s">
-        <v>677</v>
+        <v>687</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>678</v>
+        <v>688</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>679</v>
+        <v>689</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>680</v>
+        <v>690</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>681</v>
+        <v>691</v>
       </c>
       <c r="F18" s="19" t="s">
         <v>19</v>
@@ -7606,19 +7699,19 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="19" t="s">
-        <v>682</v>
+        <v>692</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>683</v>
+        <v>693</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>684</v>
+        <v>694</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>685</v>
+        <v>695</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>686</v>
+        <v>696</v>
       </c>
       <c r="F19" s="19" t="s">
         <v>19</v>
@@ -7626,59 +7719,59 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="19" t="s">
-        <v>687</v>
+        <v>697</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>688</v>
+        <v>698</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>689</v>
+        <v>699</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>690</v>
+        <v>700</v>
       </c>
       <c r="E20" s="19" t="s">
-        <v>691</v>
+        <v>701</v>
       </c>
       <c r="F20" s="19" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="19" t="s">
-        <v>692</v>
+        <v>702</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>693</v>
+        <v>703</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>694</v>
+        <v>704</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>695</v>
+        <v>705</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>696</v>
+        <v>706</v>
       </c>
       <c r="F21" s="19" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="25.5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="19" t="s">
-        <v>697</v>
+        <v>707</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>698</v>
+        <v>708</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>699</v>
+        <v>709</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>700</v>
+        <v>710</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>686</v>
+        <v>696</v>
       </c>
       <c r="F22" s="19" t="s">
         <v>19</v>
@@ -7686,19 +7779,19 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="19" t="s">
-        <v>701</v>
+        <v>711</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>702</v>
+        <v>712</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>703</v>
+        <v>713</v>
       </c>
       <c r="D23" s="19" t="s">
         <v>70</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>704</v>
+        <v>714</v>
       </c>
       <c r="F23" s="19" t="s">
         <v>21</v>
@@ -7706,19 +7799,19 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="19" t="s">
-        <v>705</v>
+        <v>715</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>706</v>
+        <v>716</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>707</v>
+        <v>717</v>
       </c>
       <c r="D24" s="19" t="s">
         <v>70</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>708</v>
+        <v>718</v>
       </c>
       <c r="F24" s="19" t="s">
         <v>21</v>
@@ -7726,13 +7819,13 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="19" t="s">
-        <v>709</v>
+        <v>719</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>710</v>
+        <v>720</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>711</v>
+        <v>721</v>
       </c>
       <c r="D25" s="19" t="s">
         <v>70</v>
@@ -7773,28 +7866,28 @@
     <col min="4" max="4" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="18" t="s">
-        <v>713</v>
+        <v>723</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>714</v>
+        <v>724</v>
       </c>
       <c r="C3" s="18" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>715</v>
+        <v>725</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
-        <v>716</v>
+        <v>726</v>
       </c>
       <c r="B4" s="19" t="s">
         <v>69</v>
@@ -7803,203 +7896,203 @@
         <v>11</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>717</v>
+        <v>727</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="19" t="s">
-        <v>716</v>
+        <v>726</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C5" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>718</v>
+        <v>728</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="19" t="s">
-        <v>716</v>
+        <v>726</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="C6" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>719</v>
+        <v>729</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="19" t="s">
-        <v>716</v>
+        <v>726</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="C7" s="19" t="s">
         <v>13</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>720</v>
+        <v>730</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="19" t="s">
-        <v>721</v>
+        <v>731</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>722</v>
+        <v>732</v>
       </c>
       <c r="C8" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>723</v>
+        <v>733</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="19" t="s">
-        <v>721</v>
+        <v>731</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>706</v>
+        <v>716</v>
       </c>
       <c r="C9" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>724</v>
+        <v>734</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="19" t="s">
-        <v>721</v>
+        <v>731</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>725</v>
+        <v>735</v>
       </c>
       <c r="C10" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>726</v>
+        <v>736</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="19" t="s">
-        <v>721</v>
+        <v>731</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>727</v>
+        <v>737</v>
       </c>
       <c r="C11" s="19" t="s">
         <v>9</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>728</v>
+        <v>738</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="19" t="s">
-        <v>721</v>
+        <v>731</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>729</v>
+        <v>739</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>9</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>730</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="25.5" x14ac:dyDescent="0.3">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="19" t="s">
-        <v>721</v>
+        <v>731</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>731</v>
+        <v>741</v>
       </c>
       <c r="C13" s="19" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>732</v>
+        <v>742</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="19" t="s">
-        <v>721</v>
+        <v>731</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>733</v>
+        <v>743</v>
       </c>
       <c r="C14" s="19" t="s">
         <v>11</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="19" t="s">
-        <v>734</v>
+        <v>744</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>735</v>
+        <v>745</v>
       </c>
       <c r="C15" s="19" t="s">
         <v>13</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>736</v>
+        <v>746</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="19" t="s">
-        <v>734</v>
+        <v>744</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>737</v>
+        <v>747</v>
       </c>
       <c r="C16" s="19" t="s">
         <v>13</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>738</v>
+        <v>748</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="19" t="s">
-        <v>734</v>
+        <v>744</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>739</v>
+        <v>749</v>
       </c>
       <c r="C17" s="19" t="s">
         <v>13</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>740</v>
+        <v>750</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="19" t="s">
-        <v>741</v>
+        <v>751</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>742</v>
+        <v>752</v>
       </c>
       <c r="C18" s="19" t="s">
         <v>13</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>743</v>
+        <v>753</v>
       </c>
     </row>
   </sheetData>

</xml_diff>